<commit_message>
test(testbed): drop study B rows from the expected DS_A spreadsheet (#368)
The RTS download for study A holds only study A's entities since the test-bed
data is one submission per study, so the expected spreadsheet loses the rows of
STUDY_B, DS_B, DAP_2 and RESEARCH_DATA_FILE_4 to _9.
The architecture doc now says the test-bed model allows exactly one study per
submission and points at the split fixture files.
</commit_message>
<xml_diff>
--- a/testbed/example_data/metadata/DS_A-downloaded.xlsx
+++ b/testbed/example_data/metadata/DS_A-downloaded.xlsx
@@ -1000,7 +1000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1094,48 +1094,6 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>EGADATASET000A</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DS_B</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>GHGAD77190331471604</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GHGAS51090952308378</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>GHGAP86954321096576</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>An interesting dataset B of complete example set</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>The complete-B dataset</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>And another Type</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>EGADATASET000B</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2466,43 +2424,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>STUDY_B</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>GHGAS51090952308378</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>EGASTUDY12346</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>A study that is the B study</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>The B Study</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>WHOLE_GENOME_SEQUENCING</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Some Institute</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2514,7 +2435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2725,294 +2646,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>RESEARCH_DATA_FILE_4</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>GHGAF77721593457161</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>GHGAX39795256829841</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>SAMPLE_2_SPECIMEN_1_FILE_4.fastq.gz</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>LANE_126</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>GHGAD77190331471604</t>
-        </is>
-      </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>FASTQ</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>EGAFILE12349</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>RESEARCH_DATA_FILE_5</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>GHGAF91562421781007</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GHGAX39795256829841</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>SAMPLE_2_SPECIMEN_1_FILE_5.fastq.gz</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>LANE_127</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>GHGAD77190331471604</t>
-        </is>
-      </c>
-      <c r="H6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>FASTQ</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>EGAFILE12350</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>RESEARCH_DATA_FILE_6</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>GHGAF63374393909479</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>GHGAX39795256829841</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>SAMPLE_2_SPECIMEN_1_FILE_6.fastq.gz</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>LANE_128</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>3</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>GHGAD77190331471604</t>
-        </is>
-      </c>
-      <c r="H7" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>FASTQ</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>EGAFILE12351</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>RESEARCH_DATA_FILE_7</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>GHGAF24594710068561</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>GHGAX39795256829841</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>SAMPLE_2_SPECIMEN_1_FILE_7.fastq.gz</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>LANE_129</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>4</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>GHGAD77190331471604</t>
-        </is>
-      </c>
-      <c r="H8" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>FASTQ</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>EGAFILE12352</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>RESEARCH_DATA_FILE_8</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>GHGAF97000461197528</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>GHGAX39795256829841</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>SAMPLE_2_SPECIMEN_1_FILE_8.fastq.gz</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>LANE_130</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>5</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>GHGAD77190331471604</t>
-        </is>
-      </c>
-      <c r="H9" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>FASTQ</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>EGAFILE12353</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>RESEARCH_DATA_FILE_9</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>GHGAF58915171737891</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>GHGAX39795256829841</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>SAMPLE_2_SPECIMEN_1_FILE_9.fastq.gz</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>LANE_131</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>6</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>GHGAD77190331471604</t>
-        </is>
-      </c>
-      <c r="H10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>FASTQ</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>EGAFILE12354</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3024,7 +2657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3165,68 +2798,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DAP_2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>GHGAP86954321096576</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>DUO:0000026</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>DAP 2</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>USER_SPECIFIC_RESTRICTION</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>http://some/other/policy</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>A Data Access Policy 2</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>This is a very strict DAP</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>NO_RESTRICTION</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>GHGAC82748725434213</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>DUO:0000004</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>EGADAP12346</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>